<commit_message>
Update: 25-26 Bahar Vize Excel verisi guncellendi
</commit_message>
<xml_diff>
--- a/25-26_Bahar_Vize.xlsx
+++ b/25-26_Bahar_Vize.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30002"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5AE7A30E-E8E7-4941-8986-34A7FA6BE2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3CCCC49-BCD3-43D6-BFDC-C8A5E1D6947E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21156,7 +21156,7 @@
         <v>447</v>
       </c>
       <c r="I577" s="111" t="s">
-        <v>293</v>
+        <v>265</v>
       </c>
       <c r="J577" s="111"/>
       <c r="K577">
@@ -21486,7 +21486,7 @@
         <v>494</v>
       </c>
       <c r="I587" s="156" t="s">
-        <v>293</v>
+        <v>265</v>
       </c>
       <c r="J587" s="136"/>
       <c r="K587" s="110">
@@ -21519,7 +21519,7 @@
         <v>494</v>
       </c>
       <c r="I588" s="156" t="s">
-        <v>293</v>
+        <v>265</v>
       </c>
       <c r="J588" s="140"/>
       <c r="K588" s="110">
@@ -22002,8 +22002,8 @@
       <c r="H607" s="484" t="s">
         <v>523</v>
       </c>
-      <c r="I607" s="165" t="s">
-        <v>258</v>
+      <c r="I607" s="111" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="608" spans="1:10" ht="15.75">

</xml_diff>

<commit_message>
Update: Excel verisi guncellendi 2026-04-09 17:34
</commit_message>
<xml_diff>
--- a/25-26_Bahar_Vize.xlsx
+++ b/25-26_Bahar_Vize.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30002"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3CCCC49-BCD3-43D6-BFDC-C8A5E1D6947E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E81CFA2E-EFAC-4D1A-A7FF-1A0AF8A27A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -943,616 +943,616 @@
     <t>PSYC2004</t>
   </si>
   <si>
+    <t>Dr. Öğr. Üyesi Melike Karatay</t>
+  </si>
+  <si>
+    <t>PSYC204</t>
+  </si>
+  <si>
+    <t>PSYC106</t>
+  </si>
+  <si>
+    <t>Dr. Özgür Çelenk</t>
+  </si>
+  <si>
+    <t>Arş. Gör. Oğuz Kaan Bulut</t>
+  </si>
+  <si>
+    <t>PSYC466</t>
+  </si>
+  <si>
+    <t>PSYC306</t>
+  </si>
+  <si>
+    <t>EKONOMİ VE FİNANS</t>
+  </si>
+  <si>
+    <t>INTF4004</t>
+  </si>
+  <si>
+    <t>Dr.Öğr.Üyesi Tuğba Baş</t>
+  </si>
+  <si>
+    <t>INTF202</t>
+  </si>
+  <si>
+    <t>Gözetmene gerek yok.</t>
+  </si>
+  <si>
+    <t>STAT284</t>
+  </si>
+  <si>
+    <t>Prof.Dr. Seda Bağdatlı Kalkan</t>
+  </si>
+  <si>
+    <t>MATH126</t>
+  </si>
+  <si>
+    <t>Dr.Öğr. Üyesi Dilara Karslıoğlu</t>
+  </si>
+  <si>
+    <t>Dr.Öğr.Üyesi Hazar Altınbaş</t>
+  </si>
+  <si>
+    <t>Dr.Öğr.Üyesi Zühal Özbay Daş</t>
+  </si>
+  <si>
+    <t>ECON454</t>
+  </si>
+  <si>
+    <t>B219</t>
+  </si>
+  <si>
+    <t>INTF357</t>
+  </si>
+  <si>
+    <t>INTF2002</t>
+  </si>
+  <si>
+    <t>F111</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Vecdi Emre Levent</t>
+  </si>
+  <si>
+    <t>ECON404</t>
+  </si>
+  <si>
+    <t>B215</t>
+  </si>
+  <si>
+    <t>INTF456</t>
+  </si>
+  <si>
+    <t>INTF3057</t>
+  </si>
+  <si>
+    <t>ECON202</t>
+  </si>
+  <si>
+    <t>INTF3002</t>
+  </si>
+  <si>
+    <t>Dr.Öğr.Üyesi Ceren İlkay Soylu</t>
+  </si>
+  <si>
+    <t>ECON356</t>
+  </si>
+  <si>
+    <t>FL2-21</t>
+  </si>
+  <si>
+    <t>ECON2032</t>
+  </si>
+  <si>
+    <t>Dr.Öğr.Üyesi Bilge Çağatay</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Bilge SERDARER KUZU</t>
+  </si>
+  <si>
+    <t>INTF306</t>
+  </si>
+  <si>
+    <t>ECON302</t>
+  </si>
+  <si>
+    <t>ECON402</t>
+  </si>
+  <si>
+    <t>ECON232</t>
+  </si>
+  <si>
+    <t>ECON458</t>
+  </si>
+  <si>
+    <t>Dr.Öğr.Üyesi Onur Yamaner</t>
+  </si>
+  <si>
+    <t>INTF2004</t>
+  </si>
+  <si>
+    <t>INTF4002</t>
+  </si>
+  <si>
+    <t>Prof. Dr. Ayben Koy</t>
+  </si>
+  <si>
+    <t>INTF3053</t>
+  </si>
+  <si>
+    <t>INTF402</t>
+  </si>
+  <si>
+    <t>İNGİLİZ DİLİ VE EDEBİYATI</t>
+  </si>
+  <si>
+    <t>FRE202</t>
+  </si>
+  <si>
+    <t>B-211</t>
+  </si>
+  <si>
+    <t>Ayla Ezgi Ozan</t>
+  </si>
+  <si>
+    <t>GER202</t>
+  </si>
+  <si>
+    <t>B-309</t>
+  </si>
+  <si>
+    <t>Vahdettin Oytun Çalışkan</t>
+  </si>
+  <si>
+    <t>ELIT106</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Başak Çün</t>
+  </si>
+  <si>
+    <t>B-310</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Berkay Üstün</t>
+  </si>
+  <si>
+    <t>ELIT112</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Serhat Uyurkulak</t>
+  </si>
+  <si>
+    <t>B-311</t>
+  </si>
+  <si>
+    <t>ELIT104</t>
+  </si>
+  <si>
+    <t>Prof. Dr. Evrim Doğan Adanur</t>
+  </si>
+  <si>
+    <t>ELIT208</t>
+  </si>
+  <si>
+    <t>ELIT214</t>
+  </si>
+  <si>
+    <t>ELIT212</t>
+  </si>
+  <si>
+    <t>B-L-01</t>
+  </si>
+  <si>
+    <t>ELIT204</t>
+  </si>
+  <si>
+    <t>ELIT314</t>
+  </si>
+  <si>
+    <t>B-409</t>
+  </si>
+  <si>
+    <t>ELIT349</t>
+  </si>
+  <si>
+    <t>B-217</t>
+  </si>
+  <si>
+    <t>ELIT337</t>
+  </si>
+  <si>
+    <t>ELIT312</t>
+  </si>
+  <si>
+    <t>B-312</t>
+  </si>
+  <si>
+    <t>ELIT304</t>
+  </si>
+  <si>
+    <t>ELIT404</t>
+  </si>
+  <si>
+    <t>ELIT402</t>
+  </si>
+  <si>
+    <t>B-314</t>
+  </si>
+  <si>
+    <t>ELIT416</t>
+  </si>
+  <si>
+    <t>B-501</t>
+  </si>
+  <si>
+    <t>SBUI</t>
+  </si>
+  <si>
+    <t>POLS468</t>
+  </si>
+  <si>
+    <t>Doç.Dr. Hazal Papuççular Kutlu</t>
+  </si>
+  <si>
+    <t>Araştırma Görevlisi Rümeysa Karagöz</t>
+  </si>
+  <si>
+    <t>POLS202</t>
+  </si>
+  <si>
+    <t>Dr. Nur Çetiner Plevne</t>
+  </si>
+  <si>
+    <t>ECON102</t>
+  </si>
+  <si>
+    <t>Dr.Öğr. Üyesi Zuhal Özbay Daş</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Hazar Altınbaş</t>
+  </si>
+  <si>
+    <t>B-315</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Ceren İlkay Soylu Küçükgöncü</t>
+  </si>
+  <si>
+    <t>STAT280</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Mehmet Gürel Tekelioğlu</t>
+  </si>
+  <si>
+    <t>Araştırma Görevlis Mehmet Emir Erdem</t>
+  </si>
+  <si>
+    <t>Araştrıma Görevlisi Esra Misem Sönmez</t>
+  </si>
+  <si>
+    <t>IR302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doç. Dr.Nihan Akıncılar Köseoğlu </t>
+  </si>
+  <si>
+    <t>HIST104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr.Öğr. Üyesi Onur Yamaner </t>
+  </si>
+  <si>
+    <t>Arş. Gör. Mehmet Emir Erdem</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Zuhal Özbay Daş</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Zeynep Kabadayı Kuşçu</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Tuğba Baş</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arş. Gör. Cem Bağlum </t>
+  </si>
+  <si>
+    <t>Dr. Öğretim Üyesi Bilge Çağatay</t>
+  </si>
+  <si>
+    <t>POLS388</t>
+  </si>
+  <si>
+    <t>B-215</t>
+  </si>
+  <si>
+    <t>Doç. Dr. Hazal Papuççular Kutlu</t>
+  </si>
+  <si>
+    <t>IR102</t>
+  </si>
+  <si>
+    <t>IR404</t>
+  </si>
+  <si>
+    <t>Doç. Dr. Nihan Akıncılar Köseoğlu</t>
+  </si>
+  <si>
+    <t>STAT240</t>
+  </si>
+  <si>
+    <t>Prof. Dr.Seda Bağdatlı Kalkan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Öğr. Üyesi Bilge Çağatay </t>
+  </si>
+  <si>
+    <t>Araştırma Görevlisi Oğuz Kaan Bulut</t>
+  </si>
+  <si>
+    <t>POLS470</t>
+  </si>
+  <si>
+    <t>Doç. Dr. Ercan Gündoğan</t>
+  </si>
+  <si>
+    <t>PSYC134</t>
+  </si>
+  <si>
+    <t>POLS304</t>
+  </si>
+  <si>
+    <t>Dr. Levent Önen</t>
+  </si>
+  <si>
+    <t>POLS354</t>
+  </si>
+  <si>
+    <t>B-219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doç.Dr. Nihan Akıncılar Köseoğlu </t>
+  </si>
+  <si>
+    <t>LAW234</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Öğr. Üyesi Saniye Sena Cabıoğlu Güler </t>
+  </si>
+  <si>
+    <t>IR204</t>
+  </si>
+  <si>
+    <t>Dr.Tuncer Beyribey</t>
+  </si>
+  <si>
+    <t>MIS</t>
+  </si>
+  <si>
+    <t>MIS102</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Ferhat Kutlu</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Dilara Karslıoğlu</t>
+  </si>
+  <si>
+    <t>MIS402</t>
+  </si>
+  <si>
+    <t>MIS208</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Birsen Özalp</t>
+  </si>
+  <si>
+    <t>MIS460</t>
+  </si>
+  <si>
+    <t>MIS206</t>
+  </si>
+  <si>
+    <t>Prof. Dr. Ceyda Aysuna Türkyılmaz</t>
+  </si>
+  <si>
+    <t>MIS104</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Cevahir Parlak</t>
+  </si>
+  <si>
+    <t>MIS354</t>
+  </si>
+  <si>
+    <t>F-204</t>
+  </si>
+  <si>
+    <t>MIS456</t>
+  </si>
+  <si>
+    <t>B-414</t>
+  </si>
+  <si>
+    <t>Prof. Dr. Erdal Şen</t>
+  </si>
+  <si>
+    <t>MIS306</t>
+  </si>
+  <si>
+    <t>MIS202</t>
+  </si>
+  <si>
+    <t>F-304</t>
+  </si>
+  <si>
+    <t>Prof. Dr. Kaya Kuru</t>
+  </si>
+  <si>
+    <t>MIS106</t>
+  </si>
+  <si>
+    <t>MIS308</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Adil Gürsel Karaçor</t>
+  </si>
+  <si>
+    <t>MIS370</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Ömer Özgür Bozkurt</t>
+  </si>
+  <si>
+    <t>ECON134</t>
+  </si>
+  <si>
+    <t>B-313</t>
+  </si>
+  <si>
+    <t>MIS204</t>
+  </si>
+  <si>
+    <t>YBS</t>
+  </si>
+  <si>
+    <t>YBS102</t>
+  </si>
+  <si>
+    <t>ECON141</t>
+  </si>
+  <si>
+    <t>Dr. Öğr. Üyesi Zühal Özbay Daş</t>
+  </si>
+  <si>
+    <t>HIST103</t>
+  </si>
+  <si>
+    <t>YBS104</t>
+  </si>
+  <si>
+    <t>F-317</t>
+  </si>
+  <si>
+    <t>YBS106</t>
+  </si>
+  <si>
+    <t>İŞLETME</t>
+  </si>
+  <si>
+    <t>STAT603</t>
+  </si>
+  <si>
+    <t>GRAD503</t>
+  </si>
+  <si>
+    <t>Doç.Dr. Elif Çaloğlu Büyükselçuk</t>
+  </si>
+  <si>
+    <t>GRAD603</t>
+  </si>
+  <si>
+    <t>MBA5014</t>
+  </si>
+  <si>
+    <t>Dr. Zeynep Kabadayı Kuşcu</t>
+  </si>
+  <si>
+    <t>MBA5020</t>
+  </si>
+  <si>
+    <t>EM553/INDR2006</t>
+  </si>
+  <si>
+    <t>Dr. Hazar Altınbaş</t>
+  </si>
+  <si>
+    <t>IISBF</t>
+  </si>
+  <si>
+    <t>MBA5026</t>
+  </si>
+  <si>
+    <t>Dr. Ceren Soylu</t>
+  </si>
+  <si>
+    <t>MBA5025</t>
+  </si>
+  <si>
+    <t>GRAD5003</t>
+  </si>
+  <si>
+    <t>Dr. Cem Savaş Aydın</t>
+  </si>
+  <si>
+    <t>MBA520</t>
+  </si>
+  <si>
+    <t>MBA512</t>
+  </si>
+  <si>
+    <t>MBA526</t>
+  </si>
+  <si>
+    <t>Dr. Melike Karatay</t>
+  </si>
+  <si>
+    <t>MBA504</t>
+  </si>
+  <si>
+    <t>Dr. Zühal Özbay Daş</t>
+  </si>
+  <si>
+    <t>SS515</t>
+  </si>
+  <si>
+    <t>F-L2-19</t>
+  </si>
+  <si>
+    <t>Dr. Serpil Başer</t>
+  </si>
+  <si>
+    <t>OB527</t>
+  </si>
+  <si>
+    <t>Dr. Petek Akman Özdemir</t>
+  </si>
+  <si>
+    <t>OB501</t>
+  </si>
+  <si>
+    <t>OB502</t>
+  </si>
+  <si>
+    <t>BA204</t>
+  </si>
+  <si>
+    <t>Dr. Tuğba Baş</t>
+  </si>
+  <si>
+    <t>INTF4004 ile</t>
+  </si>
+  <si>
+    <t>BA202</t>
+  </si>
+  <si>
+    <t>VBA</t>
+  </si>
+  <si>
+    <t>IST108</t>
+  </si>
+  <si>
+    <t>Prof. Dr. Şahamet BÜLBÜL</t>
+  </si>
+  <si>
+    <t>VBA102</t>
+  </si>
+  <si>
+    <t>MAT104</t>
+  </si>
+  <si>
     <t>Dr. Öğr. Üyesi Dilara KARSLIOĞLU</t>
-  </si>
-  <si>
-    <t>PSYC204</t>
-  </si>
-  <si>
-    <t>PSYC106</t>
-  </si>
-  <si>
-    <t>Dr. Özgür Çelenk</t>
-  </si>
-  <si>
-    <t>Arş. Gör. Oğuz Kaan Bulut</t>
-  </si>
-  <si>
-    <t>PSYC466</t>
-  </si>
-  <si>
-    <t>PSYC306</t>
-  </si>
-  <si>
-    <t>EKONOMİ VE FİNANS</t>
-  </si>
-  <si>
-    <t>INTF4004</t>
-  </si>
-  <si>
-    <t>Dr.Öğr.Üyesi Tuğba Baş</t>
-  </si>
-  <si>
-    <t>INTF202</t>
-  </si>
-  <si>
-    <t>Gözetmene gerek yok.</t>
-  </si>
-  <si>
-    <t>STAT284</t>
-  </si>
-  <si>
-    <t>Prof.Dr. Seda Bağdatlı Kalkan</t>
-  </si>
-  <si>
-    <t>MATH126</t>
-  </si>
-  <si>
-    <t>Dr.Öğr. Üyesi Dilara Karslıoğlu</t>
-  </si>
-  <si>
-    <t>Dr.Öğr.Üyesi Hazar Altınbaş</t>
-  </si>
-  <si>
-    <t>Dr.Öğr.Üyesi Zühal Özbay Daş</t>
-  </si>
-  <si>
-    <t>ECON454</t>
-  </si>
-  <si>
-    <t>B219</t>
-  </si>
-  <si>
-    <t>INTF357</t>
-  </si>
-  <si>
-    <t>INTF2002</t>
-  </si>
-  <si>
-    <t>F111</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Vecdi Emre Levent</t>
-  </si>
-  <si>
-    <t>ECON404</t>
-  </si>
-  <si>
-    <t>B215</t>
-  </si>
-  <si>
-    <t>INTF456</t>
-  </si>
-  <si>
-    <t>INTF3057</t>
-  </si>
-  <si>
-    <t>ECON202</t>
-  </si>
-  <si>
-    <t>INTF3002</t>
-  </si>
-  <si>
-    <t>Dr.Öğr.Üyesi Ceren İlkay Soylu</t>
-  </si>
-  <si>
-    <t>ECON356</t>
-  </si>
-  <si>
-    <t>FL2-21</t>
-  </si>
-  <si>
-    <t>ECON2032</t>
-  </si>
-  <si>
-    <t>Dr.Öğr.Üyesi Bilge Çağatay</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Bilge SERDARER KUZU</t>
-  </si>
-  <si>
-    <t>INTF306</t>
-  </si>
-  <si>
-    <t>ECON302</t>
-  </si>
-  <si>
-    <t>ECON402</t>
-  </si>
-  <si>
-    <t>ECON232</t>
-  </si>
-  <si>
-    <t>ECON458</t>
-  </si>
-  <si>
-    <t>Dr.Öğr.Üyesi Onur Yamaner</t>
-  </si>
-  <si>
-    <t>INTF2004</t>
-  </si>
-  <si>
-    <t>INTF4002</t>
-  </si>
-  <si>
-    <t>Prof. Dr. Ayben Koy</t>
-  </si>
-  <si>
-    <t>INTF3053</t>
-  </si>
-  <si>
-    <t>INTF402</t>
-  </si>
-  <si>
-    <t>İNGİLİZ DİLİ VE EDEBİYATI</t>
-  </si>
-  <si>
-    <t>FRE202</t>
-  </si>
-  <si>
-    <t>B-211</t>
-  </si>
-  <si>
-    <t>Ayla Ezgi Ozan</t>
-  </si>
-  <si>
-    <t>GER202</t>
-  </si>
-  <si>
-    <t>B-309</t>
-  </si>
-  <si>
-    <t>Vahdettin Oytun Çalışkan</t>
-  </si>
-  <si>
-    <t>ELIT106</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Başak Çün</t>
-  </si>
-  <si>
-    <t>B-310</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Berkay Üstün</t>
-  </si>
-  <si>
-    <t>ELIT112</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Serhat Uyurkulak</t>
-  </si>
-  <si>
-    <t>B-311</t>
-  </si>
-  <si>
-    <t>ELIT104</t>
-  </si>
-  <si>
-    <t>Prof. Dr. Evrim Doğan Adanur</t>
-  </si>
-  <si>
-    <t>ELIT208</t>
-  </si>
-  <si>
-    <t>ELIT214</t>
-  </si>
-  <si>
-    <t>ELIT212</t>
-  </si>
-  <si>
-    <t>B-L-01</t>
-  </si>
-  <si>
-    <t>ELIT204</t>
-  </si>
-  <si>
-    <t>ELIT314</t>
-  </si>
-  <si>
-    <t>B-409</t>
-  </si>
-  <si>
-    <t>ELIT349</t>
-  </si>
-  <si>
-    <t>B-217</t>
-  </si>
-  <si>
-    <t>ELIT337</t>
-  </si>
-  <si>
-    <t>ELIT312</t>
-  </si>
-  <si>
-    <t>B-312</t>
-  </si>
-  <si>
-    <t>ELIT304</t>
-  </si>
-  <si>
-    <t>ELIT404</t>
-  </si>
-  <si>
-    <t>ELIT402</t>
-  </si>
-  <si>
-    <t>B-314</t>
-  </si>
-  <si>
-    <t>ELIT416</t>
-  </si>
-  <si>
-    <t>B-501</t>
-  </si>
-  <si>
-    <t>SBUI</t>
-  </si>
-  <si>
-    <t>POLS468</t>
-  </si>
-  <si>
-    <t>Doç.Dr. Hazal Papuççular Kutlu</t>
-  </si>
-  <si>
-    <t>Araştırma Görevlisi Rümeysa Karagöz</t>
-  </si>
-  <si>
-    <t>POLS202</t>
-  </si>
-  <si>
-    <t>Dr. Nur Çetiner Plevne</t>
-  </si>
-  <si>
-    <t>ECON102</t>
-  </si>
-  <si>
-    <t>Dr.Öğr. Üyesi Zuhal Özbay Daş</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Hazar Altınbaş</t>
-  </si>
-  <si>
-    <t>B-315</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Ceren İlkay Soylu Küçükgöncü</t>
-  </si>
-  <si>
-    <t>STAT280</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Mehmet Gürel Tekelioğlu</t>
-  </si>
-  <si>
-    <t>Araştırma Görevlis Mehmet Emir Erdem</t>
-  </si>
-  <si>
-    <t>Araştrıma Görevlisi Esra Misem Sönmez</t>
-  </si>
-  <si>
-    <t>IR302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doç. Dr.Nihan Akıncılar Köseoğlu </t>
-  </si>
-  <si>
-    <t>HIST104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dr.Öğr. Üyesi Onur Yamaner </t>
-  </si>
-  <si>
-    <t>Arş. Gör. Mehmet Emir Erdem</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Zuhal Özbay Daş</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Melike Karatay</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Zeynep Kabadayı Kuşçu</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Tuğba Baş</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arş. Gör. Cem Bağlum </t>
-  </si>
-  <si>
-    <t>Dr. Öğretim Üyesi Bilge Çağatay</t>
-  </si>
-  <si>
-    <t>POLS388</t>
-  </si>
-  <si>
-    <t>B-215</t>
-  </si>
-  <si>
-    <t>Doç. Dr. Hazal Papuççular Kutlu</t>
-  </si>
-  <si>
-    <t>IR102</t>
-  </si>
-  <si>
-    <t>IR404</t>
-  </si>
-  <si>
-    <t>Doç. Dr. Nihan Akıncılar Köseoğlu</t>
-  </si>
-  <si>
-    <t>STAT240</t>
-  </si>
-  <si>
-    <t>Prof. Dr.Seda Bağdatlı Kalkan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dr. Öğr. Üyesi Bilge Çağatay </t>
-  </si>
-  <si>
-    <t>Araştırma Görevlisi Oğuz Kaan Bulut</t>
-  </si>
-  <si>
-    <t>POLS470</t>
-  </si>
-  <si>
-    <t>Doç. Dr. Ercan Gündoğan</t>
-  </si>
-  <si>
-    <t>PSYC134</t>
-  </si>
-  <si>
-    <t>POLS304</t>
-  </si>
-  <si>
-    <t>Dr. Levent Önen</t>
-  </si>
-  <si>
-    <t>POLS354</t>
-  </si>
-  <si>
-    <t>B-219</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doç.Dr. Nihan Akıncılar Köseoğlu </t>
-  </si>
-  <si>
-    <t>LAW234</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dr. Öğr. Üyesi Saniye Sena Cabıoğlu Güler </t>
-  </si>
-  <si>
-    <t>IR204</t>
-  </si>
-  <si>
-    <t>Dr.Tuncer Beyribey</t>
-  </si>
-  <si>
-    <t>MIS</t>
-  </si>
-  <si>
-    <t>MIS102</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Ferhat Kutlu</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Dilara Karslıoğlu</t>
-  </si>
-  <si>
-    <t>MIS402</t>
-  </si>
-  <si>
-    <t>MIS208</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Birsen Özalp</t>
-  </si>
-  <si>
-    <t>MIS460</t>
-  </si>
-  <si>
-    <t>MIS206</t>
-  </si>
-  <si>
-    <t>Prof. Dr. Ceyda Aysuna Türkyılmaz</t>
-  </si>
-  <si>
-    <t>MIS104</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Cevahir Parlak</t>
-  </si>
-  <si>
-    <t>MIS354</t>
-  </si>
-  <si>
-    <t>F-204</t>
-  </si>
-  <si>
-    <t>MIS456</t>
-  </si>
-  <si>
-    <t>B-414</t>
-  </si>
-  <si>
-    <t>Prof. Dr. Erdal Şen</t>
-  </si>
-  <si>
-    <t>MIS306</t>
-  </si>
-  <si>
-    <t>MIS202</t>
-  </si>
-  <si>
-    <t>F-304</t>
-  </si>
-  <si>
-    <t>Prof. Dr. Kaya Kuru</t>
-  </si>
-  <si>
-    <t>MIS106</t>
-  </si>
-  <si>
-    <t>MIS308</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Adil Gürsel Karaçor</t>
-  </si>
-  <si>
-    <t>MIS370</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Ömer Özgür Bozkurt</t>
-  </si>
-  <si>
-    <t>ECON134</t>
-  </si>
-  <si>
-    <t>B-313</t>
-  </si>
-  <si>
-    <t>MIS204</t>
-  </si>
-  <si>
-    <t>YBS</t>
-  </si>
-  <si>
-    <t>YBS102</t>
-  </si>
-  <si>
-    <t>ECON141</t>
-  </si>
-  <si>
-    <t>Dr. Öğr. Üyesi Zühal Özbay Daş</t>
-  </si>
-  <si>
-    <t>HIST103</t>
-  </si>
-  <si>
-    <t>YBS104</t>
-  </si>
-  <si>
-    <t>F-317</t>
-  </si>
-  <si>
-    <t>YBS106</t>
-  </si>
-  <si>
-    <t>İŞLETME</t>
-  </si>
-  <si>
-    <t>STAT603</t>
-  </si>
-  <si>
-    <t>GRAD503</t>
-  </si>
-  <si>
-    <t>Doç.Dr. Elif Çaloğlu Büyükselçuk</t>
-  </si>
-  <si>
-    <t>GRAD603</t>
-  </si>
-  <si>
-    <t>MBA5014</t>
-  </si>
-  <si>
-    <t>Dr. Zeynep Kabadayı Kuşcu</t>
-  </si>
-  <si>
-    <t>MBA5020</t>
-  </si>
-  <si>
-    <t>EM553/INDR2006</t>
-  </si>
-  <si>
-    <t>Dr. Hazar Altınbaş</t>
-  </si>
-  <si>
-    <t>IISBF</t>
-  </si>
-  <si>
-    <t>MBA5026</t>
-  </si>
-  <si>
-    <t>Dr. Ceren Soylu</t>
-  </si>
-  <si>
-    <t>MBA5025</t>
-  </si>
-  <si>
-    <t>GRAD5003</t>
-  </si>
-  <si>
-    <t>Dr. Cem Savaş Aydın</t>
-  </si>
-  <si>
-    <t>MBA520</t>
-  </si>
-  <si>
-    <t>MBA512</t>
-  </si>
-  <si>
-    <t>MBA526</t>
-  </si>
-  <si>
-    <t>Dr. Melike Karatay</t>
-  </si>
-  <si>
-    <t>MBA504</t>
-  </si>
-  <si>
-    <t>Dr. Zühal Özbay Daş</t>
-  </si>
-  <si>
-    <t>SS515</t>
-  </si>
-  <si>
-    <t>F-L2-19</t>
-  </si>
-  <si>
-    <t>Dr. Serpil Başer</t>
-  </si>
-  <si>
-    <t>OB527</t>
-  </si>
-  <si>
-    <t>Dr. Petek Akman Özdemir</t>
-  </si>
-  <si>
-    <t>OB501</t>
-  </si>
-  <si>
-    <t>OB502</t>
-  </si>
-  <si>
-    <t>BA204</t>
-  </si>
-  <si>
-    <t>Dr. Tuğba Baş</t>
-  </si>
-  <si>
-    <t>INTF4004 ile</t>
-  </si>
-  <si>
-    <t>BA202</t>
-  </si>
-  <si>
-    <t>VBA</t>
-  </si>
-  <si>
-    <t>IST108</t>
-  </si>
-  <si>
-    <t>Prof. Dr. Şahamet BÜLBÜL</t>
-  </si>
-  <si>
-    <t>VBA102</t>
-  </si>
-  <si>
-    <t>MAT104</t>
   </si>
   <si>
     <t>MAT106</t>
@@ -19580,7 +19580,7 @@
         <v>265</v>
       </c>
       <c r="J521" s="140" t="s">
-        <v>404</v>
+        <v>302</v>
       </c>
     </row>
     <row r="522" spans="1:10">
@@ -19609,10 +19609,10 @@
         <v>401</v>
       </c>
       <c r="I522" s="140" t="s">
+        <v>404</v>
+      </c>
+      <c r="J522" s="140" t="s">
         <v>405</v>
-      </c>
-      <c r="J522" s="140" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="523" spans="1:10">
@@ -19641,15 +19641,15 @@
         <v>401</v>
       </c>
       <c r="I523" s="140" t="s">
+        <v>406</v>
+      </c>
+      <c r="J523" s="140" t="s">
         <v>407</v>
-      </c>
-      <c r="J523" s="140" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="524" spans="1:10">
       <c r="A524" s="47" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B524" s="47">
         <v>1</v>
@@ -19658,7 +19658,7 @@
         <v>133</v>
       </c>
       <c r="D524" s="47" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E524" s="77">
         <v>46134</v>
@@ -19673,13 +19673,13 @@
         <v>401</v>
       </c>
       <c r="I524" s="140" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J524" s="140"/>
     </row>
     <row r="525" spans="1:10">
       <c r="A525" s="47" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B525" s="47">
         <v>1</v>
@@ -19703,13 +19703,13 @@
         <v>399</v>
       </c>
       <c r="I525" s="140" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J525" s="140"/>
     </row>
     <row r="526" spans="1:10">
       <c r="A526" s="47" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B526" s="47">
         <v>1</v>
@@ -19733,13 +19733,13 @@
         <v>385</v>
       </c>
       <c r="I526" s="140" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="J526" s="140"/>
     </row>
     <row r="527" spans="1:10">
       <c r="A527" s="94" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B527" s="94">
         <v>1</v>
@@ -19760,18 +19760,18 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H527" s="47" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="I527" s="140" t="s">
         <v>265</v>
       </c>
       <c r="J527" s="140" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="528" spans="1:10">
       <c r="A528" s="94" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B528" s="94">
         <v>1</v>
@@ -19792,18 +19792,18 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H528" s="47" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="I528" s="140" t="s">
         <v>293</v>
       </c>
       <c r="J528" s="140" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="529" spans="1:10">
       <c r="A529" s="47" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B529" s="47">
         <v>1</v>
@@ -19824,16 +19824,16 @@
         <v>0.63541666666666663</v>
       </c>
       <c r="H529" s="47" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="I529" s="140" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="J529" s="140"/>
     </row>
     <row r="530" spans="1:10">
       <c r="A530" s="94" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B530" s="94">
         <v>1</v>
@@ -19863,7 +19863,7 @@
     </row>
     <row r="531" spans="1:10">
       <c r="A531" s="94" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B531" s="94">
         <v>1</v>
@@ -19887,13 +19887,13 @@
         <v>243</v>
       </c>
       <c r="I531" s="140" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="J531" s="140"/>
     </row>
     <row r="532" spans="1:10">
       <c r="A532" s="94" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B532" s="94">
         <v>1</v>
@@ -19923,7 +19923,7 @@
     </row>
     <row r="533" spans="1:10">
       <c r="A533" s="47" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B533" s="47">
         <v>1</v>
@@ -19944,7 +19944,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H533" s="47" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="I533" s="140" t="s">
         <v>386</v>
@@ -19953,7 +19953,7 @@
     </row>
     <row r="534" spans="1:10">
       <c r="A534" s="47" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B534" s="47">
         <v>1</v>
@@ -19962,7 +19962,7 @@
         <v>133</v>
       </c>
       <c r="D534" s="47" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E534" s="77">
         <v>46140</v>
@@ -19974,7 +19974,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H534" s="47" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="I534" s="140" t="s">
         <v>262</v>
@@ -19983,7 +19983,7 @@
     </row>
     <row r="535" spans="1:10">
       <c r="A535" s="47" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B535" s="47">
         <v>1</v>
@@ -20004,7 +20004,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H535" s="47" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I535" s="140" t="s">
         <v>386</v>
@@ -20013,7 +20013,7 @@
     </row>
     <row r="536" spans="1:10">
       <c r="A536" s="47" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B536" s="47">
         <v>1</v>
@@ -20034,10 +20034,10 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H536" s="47" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="I536" s="140" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J536" s="140"/>
     </row>
@@ -20055,7 +20055,7 @@
     </row>
     <row r="538" spans="1:10" ht="15.75">
       <c r="A538" s="90" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B538" s="47"/>
       <c r="C538" s="47"/>
@@ -20069,7 +20069,7 @@
     </row>
     <row r="539" spans="1:10">
       <c r="A539" s="47" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B539" s="47">
         <v>1</v>
@@ -20090,16 +20090,16 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H539" s="47" t="s">
+        <v>432</v>
+      </c>
+      <c r="I539" s="473" t="s">
         <v>433</v>
-      </c>
-      <c r="I539" s="473" t="s">
-        <v>434</v>
       </c>
       <c r="J539" s="47"/>
     </row>
     <row r="540" spans="1:10">
       <c r="A540" s="47" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B540" s="47">
         <v>2</v>
@@ -20120,7 +20120,7 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H540" s="47" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="I540" s="47" t="s">
         <v>293</v>
@@ -20129,7 +20129,7 @@
     </row>
     <row r="541" spans="1:10">
       <c r="A541" s="47" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B541" s="47">
         <v>1</v>
@@ -20159,7 +20159,7 @@
     </row>
     <row r="542" spans="1:10">
       <c r="A542" s="47" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B542" s="47">
         <v>1</v>
@@ -20180,7 +20180,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H542" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="I542" s="47" t="s">
         <v>293</v>
@@ -20189,7 +20189,7 @@
     </row>
     <row r="543" spans="1:10">
       <c r="A543" s="47" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B543" s="47">
         <v>1</v>
@@ -20210,16 +20210,16 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H543" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="I543" s="47" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="J543" s="47"/>
     </row>
     <row r="544" spans="1:10">
       <c r="A544" s="47" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B544" s="47">
         <v>1</v>
@@ -20249,7 +20249,7 @@
     </row>
     <row r="545" spans="1:10">
       <c r="A545" s="47" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B545" s="47">
         <v>1</v>
@@ -20270,7 +20270,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H545" s="47" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="I545" s="47" t="s">
         <v>265</v>
@@ -20279,7 +20279,7 @@
     </row>
     <row r="546" spans="1:10">
       <c r="A546" s="47" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B546" s="47">
         <v>1</v>
@@ -20300,7 +20300,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H546" s="47" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="I546" s="47" t="s">
         <v>293</v>
@@ -20309,7 +20309,7 @@
     </row>
     <row r="547" spans="1:10">
       <c r="A547" s="47" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B547" s="47">
         <v>1</v>
@@ -20330,7 +20330,7 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H547" s="47" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I547" s="47" t="s">
         <v>325</v>
@@ -20339,7 +20339,7 @@
     </row>
     <row r="548" spans="1:10">
       <c r="A548" s="47" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B548" s="47">
         <v>1</v>
@@ -20360,16 +20360,16 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H548" s="47" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="I548" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="J548" s="47"/>
     </row>
     <row r="549" spans="1:10">
       <c r="A549" s="47" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B549" s="47">
         <v>1</v>
@@ -20378,7 +20378,7 @@
         <v>133</v>
       </c>
       <c r="D549" s="47" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="E549" s="77">
         <v>46134</v>
@@ -20393,13 +20393,13 @@
         <v>395</v>
       </c>
       <c r="I549" s="47" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="J549" s="47"/>
     </row>
     <row r="550" spans="1:10">
       <c r="A550" s="47" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B550" s="47">
         <v>1</v>
@@ -20408,7 +20408,7 @@
         <v>133</v>
       </c>
       <c r="D550" s="47" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E550" s="77">
         <v>46134</v>
@@ -20420,16 +20420,16 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H550" s="47" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="I550" s="158" t="s">
-        <v>404</v>
+        <v>433</v>
       </c>
       <c r="J550" s="47"/>
     </row>
     <row r="551" spans="1:10">
       <c r="A551" s="47" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B551" s="47">
         <v>1</v>
@@ -20450,7 +20450,7 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H551" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="I551" s="47" t="s">
         <v>265</v>
@@ -20459,7 +20459,7 @@
     </row>
     <row r="552" spans="1:10">
       <c r="A552" s="47" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B552" s="47">
         <v>1</v>
@@ -20480,7 +20480,7 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H552" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="I552" s="47" t="s">
         <v>293</v>
@@ -20489,7 +20489,7 @@
     </row>
     <row r="553" spans="1:10">
       <c r="A553" s="47" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B553" s="47">
         <v>1</v>
@@ -20498,7 +20498,7 @@
         <v>133</v>
       </c>
       <c r="D553" s="47" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="E553" s="77">
         <v>46139</v>
@@ -20510,16 +20510,16 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H553" s="47" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="I553" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="J553" s="47"/>
     </row>
     <row r="554" spans="1:10">
       <c r="A554" s="47" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B554" s="47">
         <v>1</v>
@@ -20540,16 +20540,16 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H554" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="I554" s="158" t="s">
-        <v>404</v>
+        <v>302</v>
       </c>
       <c r="J554" s="47"/>
     </row>
     <row r="555" spans="1:10">
       <c r="A555" s="47" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B555" s="47">
         <v>1</v>
@@ -20570,16 +20570,16 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H555" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="I555" s="47" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="J555" s="47"/>
     </row>
     <row r="556" spans="1:10">
       <c r="A556" s="47" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B556" s="47">
         <v>1</v>
@@ -20600,16 +20600,16 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H556" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="I556" s="47" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="J556" s="47"/>
     </row>
     <row r="557" spans="1:10">
       <c r="A557" s="47" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B557" s="47">
         <v>1</v>
@@ -20618,7 +20618,7 @@
         <v>133</v>
       </c>
       <c r="D557" s="47" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="E557" s="77">
         <v>46140</v>
@@ -20630,7 +20630,7 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H557" s="47" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="I557" s="47" t="s">
         <v>265</v>
@@ -20639,7 +20639,7 @@
     </row>
     <row r="558" spans="1:10">
       <c r="A558" s="47" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B558" s="47">
         <v>1</v>
@@ -20660,7 +20660,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H558" s="47" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="I558" s="473" t="s">
         <v>391</v>
@@ -20669,7 +20669,7 @@
     </row>
     <row r="559" spans="1:10">
       <c r="A559" s="47" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B559" s="47">
         <v>1</v>
@@ -20693,13 +20693,13 @@
         <v>393</v>
       </c>
       <c r="I559" s="47" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="J559" s="47"/>
     </row>
     <row r="560" spans="1:10">
       <c r="A560" s="47" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B560" s="47">
         <v>1</v>
@@ -20723,13 +20723,13 @@
         <v>393</v>
       </c>
       <c r="I560" s="47" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="J560" s="47"/>
     </row>
     <row r="561" spans="1:11">
       <c r="A561" s="47" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B561" s="47">
         <v>1</v>
@@ -20738,7 +20738,7 @@
         <v>133</v>
       </c>
       <c r="D561" s="47" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="E561" s="77">
         <v>46140</v>
@@ -20753,13 +20753,13 @@
         <v>393</v>
       </c>
       <c r="I561" s="47" t="s">
-        <v>404</v>
+        <v>302</v>
       </c>
       <c r="J561" s="47"/>
     </row>
     <row r="562" spans="1:11">
       <c r="A562" s="47" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B562" s="47">
         <v>1</v>
@@ -20780,7 +20780,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H562" s="47" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="I562" s="47" t="s">
         <v>256</v>
@@ -20801,7 +20801,7 @@
     </row>
     <row r="564" spans="1:11" ht="15.75">
       <c r="A564" s="90" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B564" s="47"/>
       <c r="C564" s="47"/>
@@ -20815,7 +20815,7 @@
     </row>
     <row r="565" spans="1:11">
       <c r="A565" s="47" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B565" s="47">
         <v>1</v>
@@ -20836,7 +20836,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H565" s="47" t="s">
-        <v>404</v>
+        <v>302</v>
       </c>
       <c r="I565" s="47" t="s">
         <v>293</v>
@@ -20845,7 +20845,7 @@
     </row>
     <row r="566" spans="1:11">
       <c r="A566" s="47" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B566" s="47">
         <v>1</v>
@@ -20854,7 +20854,7 @@
         <v>133</v>
       </c>
       <c r="D566" s="47" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E566" s="77">
         <v>46132</v>
@@ -20866,7 +20866,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H566" s="47" t="s">
-        <v>404</v>
+        <v>302</v>
       </c>
       <c r="I566" s="47" t="s">
         <v>258</v>
@@ -20875,7 +20875,7 @@
     </row>
     <row r="567" spans="1:11">
       <c r="A567" s="47" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B567" s="47">
         <v>1</v>
@@ -20896,7 +20896,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H567" s="47" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="I567" s="47" t="s">
         <v>293</v>
@@ -20905,7 +20905,7 @@
     </row>
     <row r="568" spans="1:11">
       <c r="A568" s="47" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B568" s="47">
         <v>1</v>
@@ -20935,7 +20935,7 @@
     </row>
     <row r="569" spans="1:11">
       <c r="A569" s="47" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B569" s="47">
         <v>1</v>
@@ -20944,7 +20944,7 @@
         <v>133</v>
       </c>
       <c r="D569" s="47" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E569" s="77">
         <v>46134</v>
@@ -20959,13 +20959,13 @@
         <v>325</v>
       </c>
       <c r="I569" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="J569" s="47"/>
     </row>
     <row r="570" spans="1:11">
       <c r="A570" s="47" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B570" s="47">
         <v>1</v>
@@ -20974,7 +20974,7 @@
         <v>133</v>
       </c>
       <c r="D570" s="47" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="E570" s="77">
         <v>46136</v>
@@ -20986,7 +20986,7 @@
         <v>0.63541666666666663</v>
       </c>
       <c r="H570" s="47" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="I570" s="47" t="s">
         <v>293</v>
@@ -20995,12 +20995,12 @@
     </row>
     <row r="572" spans="1:11">
       <c r="A572" s="122" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="573" spans="1:11" ht="15.75">
       <c r="A573" s="115" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B573" s="103">
         <v>1</v>
@@ -21033,7 +21033,7 @@
     </row>
     <row r="574" spans="1:11" ht="15.75">
       <c r="A574" s="106" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B574" s="107">
         <v>1</v>
@@ -21054,7 +21054,7 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H574" s="106" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="I574" s="118" t="s">
         <v>258</v>
@@ -21066,7 +21066,7 @@
     </row>
     <row r="575" spans="1:11" ht="15.75">
       <c r="A575" s="106" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B575" s="107">
         <v>1</v>
@@ -21087,7 +21087,7 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H575" s="106" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="I575" s="118" t="s">
         <v>258</v>
@@ -21099,7 +21099,7 @@
     </row>
     <row r="576" spans="1:11" ht="15.75">
       <c r="A576" s="111" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B576" s="103">
         <v>1</v>
@@ -21120,7 +21120,7 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H576" s="111" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="I576" s="111" t="s">
         <v>49</v>
@@ -21132,7 +21132,7 @@
     </row>
     <row r="577" spans="1:11" ht="15.75">
       <c r="A577" s="111" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B577" s="103">
         <v>1</v>
@@ -21153,7 +21153,7 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H577" s="111" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="I577" s="111" t="s">
         <v>265</v>
@@ -21165,7 +21165,7 @@
     </row>
     <row r="578" spans="1:11" ht="15.75">
       <c r="A578" s="111" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B578" s="103">
         <v>1</v>
@@ -21174,7 +21174,7 @@
         <v>133</v>
       </c>
       <c r="D578" s="111" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="E578" s="112">
         <v>46134</v>
@@ -21186,10 +21186,10 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="H578" s="111" t="s">
+        <v>476</v>
+      </c>
+      <c r="I578" s="82" t="s">
         <v>477</v>
-      </c>
-      <c r="I578" s="82" t="s">
-        <v>478</v>
       </c>
       <c r="J578" s="111"/>
       <c r="K578">
@@ -21198,7 +21198,7 @@
     </row>
     <row r="579" spans="1:11" ht="15.75">
       <c r="A579" s="111" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B579" s="103">
         <v>1</v>
@@ -21219,7 +21219,7 @@
         <v>0.82291666666666663</v>
       </c>
       <c r="H579" s="111" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="I579" s="111" t="s">
         <v>49</v>
@@ -21231,7 +21231,7 @@
     </row>
     <row r="580" spans="1:11" ht="15.75">
       <c r="A580" s="111" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B580" s="103">
         <v>1</v>
@@ -21252,7 +21252,7 @@
         <v>0.71875</v>
       </c>
       <c r="H580" s="111" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="I580" s="111" t="s">
         <v>49</v>
@@ -21264,7 +21264,7 @@
     </row>
     <row r="581" spans="1:11" ht="15.75">
       <c r="A581" s="111" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B581" s="103">
         <v>1</v>
@@ -21285,7 +21285,7 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H581" s="111" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="I581" s="111" t="s">
         <v>49</v>
@@ -21297,7 +21297,7 @@
     </row>
     <row r="582" spans="1:11" ht="15.75">
       <c r="A582" s="141" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B582" s="142">
         <v>1</v>
@@ -21318,7 +21318,7 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="H582" s="141" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="I582" s="156" t="s">
         <v>293</v>
@@ -21330,7 +21330,7 @@
     </row>
     <row r="583" spans="1:11" ht="15.75">
       <c r="A583" s="130" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B583" s="131">
         <v>1</v>
@@ -21351,7 +21351,7 @@
         <v>0.71875</v>
       </c>
       <c r="H583" s="130" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="I583" s="111" t="s">
         <v>49</v>
@@ -21363,7 +21363,7 @@
     </row>
     <row r="584" spans="1:11" ht="15.75">
       <c r="A584" s="130" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B584" s="131">
         <v>1</v>
@@ -21384,7 +21384,7 @@
         <v>0.86458333333333337</v>
       </c>
       <c r="H584" s="130" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="I584" s="156" t="s">
         <v>293</v>
@@ -21396,7 +21396,7 @@
     </row>
     <row r="585" spans="1:11" ht="15.75">
       <c r="A585" s="130" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B585" s="131">
         <v>1</v>
@@ -21417,7 +21417,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="H585" s="130" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="I585" s="156" t="s">
         <v>325</v>
@@ -21429,7 +21429,7 @@
     </row>
     <row r="586" spans="1:11" ht="15.75">
       <c r="A586" s="130" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B586" s="131">
         <v>1</v>
@@ -21438,7 +21438,7 @@
         <v>133</v>
       </c>
       <c r="D586" s="130" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E586" s="132">
         <v>46132</v>
@@ -21450,7 +21450,7 @@
         <v>0.71875</v>
       </c>
       <c r="H586" s="130" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="I586" s="111" t="s">
         <v>49</v>
@@ -21462,7 +21462,7 @@
     </row>
     <row r="587" spans="1:11" ht="15.75">
       <c r="A587" s="136" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B587" s="137">
         <v>1</v>
@@ -21483,7 +21483,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="H587" s="136" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="I587" s="156" t="s">
         <v>265</v>
@@ -21495,7 +21495,7 @@
     </row>
     <row r="588" spans="1:11" ht="15.75">
       <c r="A588" s="120" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B588" s="74">
         <v>1</v>
@@ -21516,7 +21516,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="H588" s="136" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="I588" s="156" t="s">
         <v>265</v>
@@ -21528,7 +21528,7 @@
     </row>
     <row r="589" spans="1:11" ht="15.75">
       <c r="A589" s="118" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B589" s="74">
         <v>1</v>
@@ -21554,7 +21554,7 @@
     </row>
     <row r="590" spans="1:11" ht="15.75">
       <c r="A590" s="126" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B590" s="127">
         <v>1</v>
@@ -21575,10 +21575,10 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="H590" s="121" t="s">
+        <v>497</v>
+      </c>
+      <c r="I590" s="114" t="s">
         <v>498</v>
-      </c>
-      <c r="I590" s="114" t="s">
-        <v>499</v>
       </c>
       <c r="J590" s="114"/>
       <c r="K590">
@@ -21587,7 +21587,7 @@
     </row>
     <row r="591" spans="1:11" ht="15.75">
       <c r="A591" s="114" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B591" s="115">
         <v>1</v>
@@ -21608,7 +21608,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H591" s="111" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="I591" s="111" t="s">
         <v>49</v>
@@ -21620,12 +21620,12 @@
     </row>
     <row r="593" spans="1:10" ht="15.75">
       <c r="A593" s="90" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="594" spans="1:10" ht="15.75">
       <c r="A594" s="145" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B594" s="146">
         <v>1</v>
@@ -21646,7 +21646,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H594" s="153" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="I594" s="118" t="s">
         <v>258</v>
@@ -21655,7 +21655,7 @@
     </row>
     <row r="595" spans="1:10" ht="15.75">
       <c r="A595" s="149" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B595" s="150">
         <v>1</v>
@@ -21664,7 +21664,7 @@
         <v>133</v>
       </c>
       <c r="D595" s="150" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E595" s="151">
         <v>46136</v>
@@ -21685,7 +21685,7 @@
     </row>
     <row r="596" spans="1:10" ht="15.75">
       <c r="A596" s="149" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B596" s="150">
         <v>1</v>
@@ -21694,7 +21694,7 @@
         <v>133</v>
       </c>
       <c r="D596" s="150" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E596" s="151">
         <v>46134</v>
@@ -21706,7 +21706,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="H596" s="154" t="s">
-        <v>302</v>
+        <v>505</v>
       </c>
       <c r="I596" s="118" t="s">
         <v>258</v>
@@ -21724,7 +21724,7 @@
         <v>133</v>
       </c>
       <c r="D597" s="150" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E597" s="151">
         <v>46139</v>
@@ -21736,7 +21736,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="H597" s="154" t="s">
-        <v>302</v>
+        <v>505</v>
       </c>
       <c r="I597" s="158" t="s">
         <v>507</v>
@@ -21771,7 +21771,7 @@
         <v>0.76041666666666663</v>
       </c>
       <c r="H599" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="I599" t="s">
         <v>510</v>
@@ -21866,7 +21866,7 @@
     </row>
     <row r="603" spans="1:10">
       <c r="A603" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B603">
         <v>1</v>
@@ -21988,7 +21988,7 @@
         <v>133</v>
       </c>
       <c r="D607" s="481" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="E607" s="482">
         <v>46136</v>
@@ -22017,7 +22017,7 @@
         <v>133</v>
       </c>
       <c r="D608" s="488" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E608" s="489">
         <v>46136</v>
@@ -22058,7 +22058,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="H609" s="484" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="I609" s="165" t="s">
         <v>258</v>

</xml_diff>